<commit_message>
Phase 2 (wip): hybrid retrieval, grounded answers with citations, tests
- rag: page-bounded chunking (heading-aware, exact offsets), bge-m3 -> Qdrant (embedded),
  BM25, RRF, bge-reranker; every stage + timings returned; retrieval_relevance for the router
- KB API: documents, index, remove, search (ledger stores query hash only), demo corpus seed
- Chat: attachments / knowledge-base grounding, numbered sources, citation validity check
- PDFium serialised behind one lock (found a real access-violation race)
- Text normalisation + running header/footer removal (pipeline ingest-v2)
- scripts/phase2_check.py: measured run on real models -> metrics/phase2_check.json
- 29 new tests (real OCR, fake embedder/reranker), 73 total

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seed/sheets/cml_thickness_log.xlsx
+++ b/seed/sheets/cml_thickness_log.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="CML log" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CML log" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>